<commit_message>
Link Golden Excel contents to schema reconciliation
</commit_message>
<xml_diff>
--- a/docs/resources/files/GE-ISI_Master_v2_25Aug26.xlsx
+++ b/docs/resources/files/GE-ISI_Master_v2_25Aug26.xlsx
@@ -75,7 +75,7 @@
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="204">
+  <fonts count="205">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -1258,6 +1258,13 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="96">
     <fill>
@@ -2383,10 +2390,11 @@
       </bottom>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32"/>
+    <xf numFmtId="0" fontId="204" fillId="0" borderId="32"/>
   </cellStyleXfs>
-  <cellXfs count="538">
+  <cellXfs count="539">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3641,9 +3649,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="203" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="204" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
@@ -30840,7 +30850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:J111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.02734375" customWidth="1" style="422" min="1" max="1"/>
@@ -32778,6 +32788,28 @@
       <c r="D109" s="243" t="n"/>
       <c r="E109" s="243" t="n"/>
       <c r="F109" s="243" t="n"/>
+    </row>
+    <row r="111" ht="30" customHeight="1" s="422">
+      <c r="A111" s="367" t="inlineStr">
+        <is>
+          <t>6-1</t>
+        </is>
+      </c>
+      <c r="B111" s="538" t="inlineStr">
+        <is>
+          <t>Schema 50 Reconciliation</t>
+        </is>
+      </c>
+      <c r="C111" s="538" t="inlineStr">
+        <is>
+          <t>▶</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>50-table reconciliation, verified schema definitions, and unresolved slots</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A11:D59"/>
@@ -32885,6 +32917,8 @@
     <hyperlink ref="B58" location="'Video Collateral Library'!A1" display="Video Collateral Library"/>
     <hyperlink ref="A59" location="'UIX Audit Record'!A1" display="5-14"/>
     <hyperlink ref="B59" location="'UIX Audit Record'!A1" display="UIX Audit Record"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0"/>
@@ -46446,7 +46480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D75"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.9921875" customWidth="1" style="422" min="1" max="1"/>
@@ -47536,10 +47570,36 @@
       <c r="C75" s="302" t="n"/>
       <c r="D75" s="302" t="n"/>
     </row>
+    <row r="77" ht="30" customHeight="1" s="422">
+      <c r="A77" s="302" t="inlineStr">
+        <is>
+          <t>6-1</t>
+        </is>
+      </c>
+      <c r="B77" s="538" t="inlineStr">
+        <is>
+          <t>Schema 50 Reconciliation</t>
+        </is>
+      </c>
+      <c r="C77" s="538" t="inlineStr">
+        <is>
+          <t>▶</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>50-table reconciliation, verified schema definitions, and unresolved slots</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B60:C60"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>